<commit_message>
fix: normalize WA phone number to international format in BaileysService
</commit_message>
<xml_diff>
--- a/resources/templates/import_siswa.xlsx
+++ b/resources/templates/import_siswa.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="33">
   <si>
     <t>NISN</t>
   </si>
@@ -105,6 +105,15 @@
   </si>
   <si>
     <t>- Hanya siswa dengan rombel KJJ yang akan diimport</t>
+  </si>
+  <si>
+    <t>No. Wali</t>
+  </si>
+  <si>
+    <t>081234567891</t>
+  </si>
+  <si>
+    <t>No. Wali = nomor HP orang tua/wali</t>
   </si>
 </sst>
 </file>
@@ -494,7 +503,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="true" style="0"/>
@@ -511,7 +520,7 @@
     <col min="12" max="12" width="14" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -548,8 +557,11 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -586,47 +598,53 @@
       <c r="L2" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:12">
+      <c r="M2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="L3"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:13">
       <c r="L4"/>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:13">
       <c r="L5"/>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:13">
       <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:13">
       <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:13">
       <c r="A15" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:13">
       <c r="A16" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:13">
       <c r="A17" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:13">
       <c r="A18" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:12">
+      <c r="M18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" s="3" t="s">
         <v>29</v>
       </c>

</xml_diff>